<commit_message>
Deployed 9657fe1 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/NSI_Terminale/Nouveau Feuille de calcul Microsoft Excel.xlsx
+++ b/NSI_Terminale/Nouveau Feuille de calcul Microsoft Excel.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\--- LYCEE ---\ENSEIGNEMENT_G\docs\NSI_Terminale\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8358287D-28DC-4428-AE68-806AE03D03D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0920E6EF-CE21-48D2-ACFA-2D714B8FBE24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>SD</t>
   </si>
@@ -33,9 +33,6 @@
     <t>POO</t>
   </si>
   <si>
-    <t>Listes / Files / Piles / Dictionnaires</t>
-  </si>
-  <si>
     <t>Arbres</t>
   </si>
   <si>
@@ -51,9 +48,6 @@
     <t>Langage SQL</t>
   </si>
   <si>
-    <t>ARSE</t>
-  </si>
-  <si>
     <t>SoC</t>
   </si>
   <si>
@@ -63,40 +57,43 @@
     <t>Routage</t>
   </si>
   <si>
-    <t>Sécu communication</t>
-  </si>
-  <si>
-    <t>LP</t>
-  </si>
-  <si>
     <t>Calculabilité / décidabilité</t>
   </si>
   <si>
     <t>Récursivite</t>
   </si>
   <si>
-    <t>Modularité</t>
-  </si>
-  <si>
-    <t>Paradigmes de prog</t>
-  </si>
-  <si>
-    <t>Mise au point pg</t>
-  </si>
-  <si>
-    <t>AL</t>
-  </si>
-  <si>
-    <t>Algos AB/ABR</t>
-  </si>
-  <si>
-    <t>Algos Graphes</t>
-  </si>
-  <si>
     <t>Prog dynamique</t>
   </si>
   <si>
     <t>Recherche textuelle</t>
+  </si>
+  <si>
+    <t>Dictionnaires</t>
+  </si>
+  <si>
+    <t>Listes / Files / Piles /</t>
+  </si>
+  <si>
+    <t>PROG</t>
+  </si>
+  <si>
+    <t>Pratiques de programmation</t>
+  </si>
+  <si>
+    <t>ALG</t>
+  </si>
+  <si>
+    <t>Diviser pour régner</t>
+  </si>
+  <si>
+    <t>AM</t>
+  </si>
+  <si>
+    <t>Autour de Gnu Linux</t>
+  </si>
+  <si>
+    <t>Cryptographie</t>
   </si>
 </sst>
 </file>
@@ -414,159 +411,118 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A4:B22"/>
+  <dimension ref="A4:E21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>0</v>
       </c>
       <c r="B5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>13</v>
-      </c>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>13</v>
-      </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
       <c r="B21" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B22" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>